<commit_message>
Re-run sample run. Tweaks for better run.
</commit_message>
<xml_diff>
--- a/sample-data/sample-run/Tech Review.xlsx
+++ b/sample-data/sample-run/Tech Review.xlsx
@@ -39,7 +39,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -54,6 +54,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
@@ -88,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -109,6 +114,15 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -476,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -552,24 +566,24 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>4. Selected Ultimate Integrity</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>'Loss Selection' no extreme outlier ultimates</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>1 period(s) &gt; 10.0x median (1,539,016)</t>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>'Loss Selection' IBNR &gt;= 0</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Below tolerance in periods: ['2002']</t>
         </is>
       </c>
     </row>
@@ -586,12 +600,12 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>'Count Selection' IBNR &gt;= 0</t>
+          <t>'Loss Selection' no extreme outlier ultimates</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Slight negatives (within tolerance) periods: ['2005', '2006', '2007', '2012', '2014', '2017', '2022']</t>
+          <t>1 period(s) &gt; 10.0x median (1,523,948)</t>
         </is>
       </c>
     </row>
@@ -608,12 +622,12 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>'Count Selection' no extreme outlier ultimates</t>
+          <t>'Count Selection' IBNR &gt;= 0</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>1 period(s) &gt; 10.0x median (346)</t>
+          <t>Slight negatives (within tolerance) periods: ['2005', '2006', '2007', '2012', '2014', '2017', '2022']</t>
         </is>
       </c>
     </row>
@@ -625,17 +639,17 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>6. Sel - Sheet Consistency</t>
+          <t>4. Selected Ultimate Integrity</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Sel - sheets present</t>
+          <t>'Count Selection' no extreme outlier ultimates</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
+          <t>1 period(s) &gt; 10.0x median (346)</t>
         </is>
       </c>
     </row>
@@ -647,12 +661,12 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>7. X-to-Ult Triangles</t>
+          <t>6. Sel - Sheet Consistency</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>X-to-Ult triangles</t>
+          <t>Sel - sheets present</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -669,12 +683,12 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>8. Average IBNR / Unpaid</t>
+          <t>7. X-to-Ult Triangles</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Average IBNR has data</t>
+          <t>X-to-Ult triangles</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -696,7 +710,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Average Unpaid has data</t>
+          <t>Average IBNR has data</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -713,12 +727,12 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>9. Diagnostics</t>
+          <t>8. Average IBNR / Unpaid</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Diagnostics</t>
+          <t>Average Unpaid has data</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -735,12 +749,12 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>10. CL Triangle Integrity</t>
+          <t>9. Diagnostics</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>CL triangles present</t>
+          <t>Diagnostics</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -757,12 +771,12 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>11. Development Factors</t>
+          <t>10. CL Triangle Integrity</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Development factor checks</t>
+          <t>CL triangles present</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -779,17 +793,17 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>12. Paid-to-Incurred Raw Data</t>
+          <t>11. Development Factors</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Paid and Incurred present</t>
+          <t>Development factor checks</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>One or both missing — skipping</t>
+          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
         </is>
       </c>
     </row>
@@ -801,17 +815,17 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>13. Case Reserve Reasonableness</t>
+          <t>12. Paid-to-Incurred Raw Data</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Case reserves check</t>
+          <t>Paid and Incurred present</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Incurred Loss and/or Paid Loss missing — skipping</t>
+          <t>One or both missing — skipping</t>
         </is>
       </c>
     </row>
@@ -823,17 +837,17 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>14. Closure Rate Checks</t>
+          <t>13. Case Reserve Reasonableness</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Closure rate checks</t>
+          <t>Case reserves check</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Reported Count and/or Closed Count missing — skipping</t>
+          <t>Incurred Loss and/or Paid Loss missing — skipping</t>
         </is>
       </c>
     </row>
@@ -845,15 +859,37 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
+          <t>14. Closure Rate Checks</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Closure rate checks</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Reported Count and/or Closed Count missing — skipping</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
           <t>15. Severity / Frequency Trends</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>Trend checks</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Diagnostics sheet missing — skipping</t>
         </is>
@@ -902,44 +938,44 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
         <is>
           <t>1. Structure</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="9" t="inlineStr">
         <is>
           <t>File readable</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="D2" s="10" t="inlineStr">
         <is>
           <t>15 sheets</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>1. Structure</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>Measure sheets present</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="10" t="inlineStr">
         <is>
           <t>Loss Selection, Count Selection</t>
         </is>
@@ -990,209 +1026,209 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>1. Structure</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>No duplicate sheet names</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr"/>
+      <c r="D6" s="10" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>2. Period Consistency</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>All measure sheets same periods</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>25 periods</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>2. Period Consistency</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>Period sequence (non-integer — consecutive check skipped)</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>25 periods</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>3. Current Age / Maturity</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>All current ages &gt; 0</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr"/>
+      <c r="D9" s="10" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>3. Current Age / Maturity</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>All current ages multiples of 12</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>11-month development pattern detected (ages 11, 23, 35, ...) — valid</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>3. Current Age / Maturity</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>Max current age within range</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="10" t="inlineStr">
         <is>
           <t>287</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>3. Current Age / Maturity</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>Min current age &gt;= 11</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>3. Current Age / Maturity</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>Maturity ordering (non-integer periods — order check skipped)</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr"/>
+      <c r="D13" s="10" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>4. Selected Ultimate Integrity</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>'Loss Selection' no null Selected Ultimates</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr"/>
+      <c r="D14" s="10" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>4. Selected Ultimate Integrity</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>'Loss Selection' all Selected Ultimates &gt; 0</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr"/>
+      <c r="D15" s="10" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1205,7 +1241,11 @@
           <t>'Loss Selection' IBNR &gt;= 0</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr"/>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Below tolerance in periods: ['2002']</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1225,45 +1265,45 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>1 period(s) &gt; 10.0x median (1,539,016)</t>
+          <t>1 period(s) &gt; 10.0x median (1,523,948)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>4. Selected Ultimate Integrity</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>'Count Selection' no null Selected Ultimates</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr"/>
+      <c r="D18" s="10" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>4. Selected Ultimate Integrity</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t>'Count Selection' all Selected Ultimates &gt; 0</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr"/>
+      <c r="D19" s="10" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">

</xml_diff>